<commit_message>
feat(efactura): grupa «Diverse (import e-Factura)» pentru cardurile fara grupa; potrivirea dupa aceeasi normalizare ca la scriere si scrisa dupa ROWN
- FIX: MATCH_KIND avea 10 caractere si «denumire-normalizata» pica TACUT cu ORA-12899 (12 potriviri pierdute) -> coloana largita la 30
- FIX: potrivirea nu-si gasea propriul card cind factura avea spatii duble sau ghilimele -> pas nou pe db_text
- FIX: potrivirile se scriu dupa numarul rindului (denumirea din baza are ? in loc de diacritice)
- rapoartele HTML si Excel actualizate: toate cele 352 de pozitii au card

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Partner/EFACTURA_IMPORT_14-09-2026.xlsx
+++ b/docs/Partner/EFACTURA_IMPORT_14-09-2026.xlsx
@@ -10,12 +10,14 @@
     <sheet name="0. Sumar" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="1. Contragenti" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2. Carduri marfa" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="3. Documente 1209" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="3. Grupa Diverse" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="4. Documente 1209" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1. Contragenti'!$A$1:$E$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. Carduri marfa'!$A$1:$F$238</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3. Documente 1209'!$A$1:$L$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3. Grupa Diverse'!$A$1:$D$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4. Documente 1209'!$A$1:$L$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -34,14 +36,14 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
-      <sz val="13"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +60,11 @@
         <fgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF9C3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -71,13 +78,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,10 +451,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="54" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -478,7 +486,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EFactura_639250048292811215.xml (47 facturi primite, 352 pozitii)</t>
+          <t>EFactura_639250048292811215.xml — 47 facturi primite, 352 pozitii</t>
         </is>
       </c>
     </row>
@@ -499,7 +507,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Carduri de marfa create (TMS_UNIVERS TIP P)</t>
+          <t>Carduri de marfa create (TMS_UNIVERS TIP P + TMS_MPT_TVR)</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -509,7 +517,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">   din ele active</t>
+          <t xml:space="preserve">   active</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -519,7 +527,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">   din ele arhivate ca duplicate</t>
+          <t xml:space="preserve">   arhivate ca duplicate</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -529,21 +537,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Legaturi la grupe de marfuri (TMS_SYSGRP)</t>
+          <t>Carduri legate la grupe de marfuri (TMS_SYSGRP)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>154</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Carduri de servicii, intentionat fara grupa</t>
+          <t>Grupa noua «Diverse (import e-Factura)» 274/257</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11">
@@ -573,19 +581,15 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Verificare: suma document = suma factura</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>47 din 47</t>
-        </is>
-      </c>
+          <t>VERIFICARI DUPA INSERARE</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Verificare: nr. rinduri document = nr. pozitii factura</t>
+          <t>Suma document = suma factura</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -597,12 +601,36 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Verificare: antet DT 2171 / CT 5211 / depozit 1 / furnizor</t>
+          <t>Nr. rinduri = nr. pozitii</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
           <t>47 din 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Antet DT 2171 / CT 5211 / depozit 1 / furnizor</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>47 din 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Pozitii cu card de marfa in documente</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>352 din 352</t>
         </is>
       </c>
     </row>
@@ -620,7 +648,7 @@
   <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -630,7 +658,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>COD (una.md)</t>
+          <t>COD</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -893,8 +921,8 @@
     <col width="64" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -955,7 +983,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>274/133/0/0/0</t>
+          <t>274/133</t>
         </is>
       </c>
     </row>
@@ -985,7 +1013,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>274/133/0/0/0</t>
+          <t>274/133</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1043,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>278/0/0/0/0</t>
+          <t>278/0</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1073,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>278/0/0/0/0</t>
+          <t>278/0</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1103,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>274/201/0/0/0</t>
+          <t>274/201</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1133,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>274/61/0/0/0</t>
+          <t>274/61</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1163,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>283/22/0/0/0</t>
+          <t>283/22</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1193,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>274/98/0/0/0</t>
+          <t>274/98</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1223,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>274/8/0/0/0</t>
+          <t>274/8</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1253,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>274/77/0/0/0</t>
+          <t>274/77</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1283,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>274/77/0/0/0</t>
+          <t>274/77</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1313,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>274/77/0/0/0</t>
+          <t>274/77</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1343,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>274/0/0/0/0</t>
+          <t>274/0</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1373,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>274/224/0/0/0</t>
+          <t>274/224</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1403,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>274/29/0/0/0</t>
+          <t>274/29</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1433,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>274/33/0/0/0</t>
+          <t>274/33</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1463,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>274/21/0/0/0</t>
+          <t>274/21</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1493,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>274/0/0/0/0</t>
+          <t>274/0</t>
         </is>
       </c>
     </row>
@@ -1495,7 +1523,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>274/8/0/0/0</t>
+          <t>274/8</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1575,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>274/206/0/0/0</t>
+          <t>274/206</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1605,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>274/37/0/0/0</t>
+          <t>274/37</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1635,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>283/75/0/0/0</t>
+          <t>283/75</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1665,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>276/56/0/0/0</t>
+          <t>276/56</t>
         </is>
       </c>
     </row>
@@ -1667,7 +1695,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>274/162/0/0/0</t>
+          <t>274/162</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1725,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>274/162/0/0/0</t>
+          <t>274/162</t>
         </is>
       </c>
     </row>
@@ -1727,7 +1755,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>274/162/0/0/0</t>
+          <t>274/162</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1785,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>281/35/0/0/0</t>
+          <t>281/35</t>
         </is>
       </c>
     </row>
@@ -1787,7 +1815,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>274/164/0/0/0</t>
+          <t>274/164</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1845,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>274/33/0/0/0</t>
+          <t>274/33</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1875,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>274/62/0/0/0</t>
+          <t>274/62</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1905,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>274/111/0/0/0</t>
+          <t>274/111</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1935,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>283/52/0/0/0</t>
+          <t>283/52</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1965,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>283/52/0/0/0</t>
+          <t>283/52</t>
         </is>
       </c>
     </row>
@@ -1967,7 +1995,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>283/52/0/0/0</t>
+          <t>283/52</t>
         </is>
       </c>
     </row>
@@ -1997,7 +2025,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>283/52/0/0/0</t>
+          <t>283/52</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2055,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>277/13/0/0/0</t>
+          <t>277/13</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2085,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>277/13/0/0/0</t>
+          <t>277/13</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2137,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>283/3/0/0/0</t>
+          <t>283/3</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2167,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>283/3/0/0/0</t>
+          <t>283/3</t>
         </is>
       </c>
     </row>
@@ -2169,7 +2197,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>283/3/0/0/0</t>
+          <t>283/3</t>
         </is>
       </c>
     </row>
@@ -2199,7 +2227,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>283/5/0/0/0</t>
+          <t>283/5</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2257,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>274/251/0/0/0</t>
+          <t>274/251</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2287,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>276/95/0/0/0</t>
+          <t>276/95</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2317,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>276/95/0/0/0</t>
+          <t>276/95</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2347,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>276/95/0/0/0</t>
+          <t>276/95</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2377,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>276/95/0/0/0</t>
+          <t>276/95</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2407,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>276/95/0/0/0</t>
+          <t>276/95</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2437,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>283/73/0/0/0</t>
+          <t>283/73</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2467,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>283/73/0/0/0</t>
+          <t>283/73</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2497,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>283/73/0/0/0</t>
+          <t>283/73</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2527,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>274/92/0/0/0</t>
+          <t>274/92</t>
         </is>
       </c>
     </row>
@@ -2529,7 +2557,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>274/92/0/0/0</t>
+          <t>274/92</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2587,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>274/250/0/0/0</t>
+          <t>274/250</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2639,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>274/250/0/0/0</t>
+          <t>274/250</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2669,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>274/86/0/0/0</t>
+          <t>274/86</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2699,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>274/42/0/0/0</t>
+          <t>274/42</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2729,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>274/77/0/0/0</t>
+          <t>274/77</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2759,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>274/77/0/0/0</t>
+          <t>274/77</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2789,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>274/77/0/0/0</t>
+          <t>274/77</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2819,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>274/77/0/0/0</t>
+          <t>274/77</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2849,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>281/35/0/0/0</t>
+          <t>281/35</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2879,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>277/13/0/0/0</t>
+          <t>277/13</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2909,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>274/0/0/0/0</t>
+          <t>274/0</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2939,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>276/82/0/0/0</t>
+          <t>276/82</t>
         </is>
       </c>
     </row>
@@ -2985,7 +3013,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>274/207/0/0/0</t>
+          <t>274/207</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3065,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>274/21/0/0/0</t>
+          <t>274/21</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3095,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>274/136/0/0/0</t>
+          <t>274/136</t>
         </is>
       </c>
     </row>
@@ -3119,7 +3147,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>274/86/0/0/0</t>
+          <t>274/86</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3177,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>283/75/0/0/0</t>
+          <t>283/75</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3207,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>281/35/0/0/0</t>
+          <t>281/35</t>
         </is>
       </c>
     </row>
@@ -3206,30 +3234,34 @@
       <c r="F79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" t="n">
+      <c r="A80" s="4" t="n">
         <v>540810</v>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B80" s="4" t="inlineStr">
         <is>
           <t>Cloud Baza Storno</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>buc.</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>activ</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>— serviciu, fara grupa</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr"/>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>buc.</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>activ</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>Diverse (import e-Factura)</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>274/257</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3257,7 +3289,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>274/77/0/0/0</t>
+          <t>274/77</t>
         </is>
       </c>
     </row>
@@ -3309,7 +3341,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>278/0/0/0/0</t>
+          <t>278/0</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3393,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>281/38/0/0/0</t>
+          <t>281/38</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3423,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>274/133/0/0/0</t>
+          <t>274/133</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3453,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>274/17/0/0/0</t>
+          <t>274/17</t>
         </is>
       </c>
     </row>
@@ -3473,7 +3505,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>283/75/0/0/0</t>
+          <t>283/75</t>
         </is>
       </c>
     </row>
@@ -3525,7 +3557,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>274/33/0/0/0</t>
+          <t>274/33</t>
         </is>
       </c>
     </row>
@@ -3552,56 +3584,64 @@
       <c r="F92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" t="n">
+      <c r="A93" s="4" t="n">
         <v>540823</v>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B93" s="4" t="inlineStr">
         <is>
           <t>Servicii de certificare a cheilor publice pentru semnatura electronica calificata cu termen de valabilitate 2 an</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C93" s="4" t="inlineStr">
         <is>
           <t>serv.</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>activ</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>— serviciu, fara grupa</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr"/>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>activ</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>Diverse (import e-Factura)</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>274/257</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" t="n">
+      <c r="A94" s="4" t="n">
         <v>540824</v>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B94" s="4" t="inlineStr">
         <is>
           <t>Dispozitiv criptografic-ePass 2003</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>buc.</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>activ</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>— serviciu, fara grupa</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr"/>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>buc.</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>activ</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="inlineStr">
+        <is>
+          <t>Diverse (import e-Factura)</t>
+        </is>
+      </c>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>274/257</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n">
@@ -3651,7 +3691,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>274/33/0/0/0</t>
+          <t>274/33</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3743,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>274/0/0/0/0</t>
+          <t>274/0</t>
         </is>
       </c>
     </row>
@@ -3733,7 +3773,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>274/62/0/0/0</t>
+          <t>274/62</t>
         </is>
       </c>
     </row>
@@ -3763,7 +3803,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>274/111/0/0/0</t>
+          <t>274/111</t>
         </is>
       </c>
     </row>
@@ -3793,7 +3833,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>283/21/0/0/0</t>
+          <t>283/21</t>
         </is>
       </c>
     </row>
@@ -3823,7 +3863,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>277/13/0/0/0</t>
+          <t>277/13</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3915,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>274/201/0/0/0</t>
+          <t>274/201</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3967,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>278/0/0/0/0</t>
+          <t>278/0</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3997,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>278/0/0/0/0</t>
+          <t>278/0</t>
         </is>
       </c>
     </row>
@@ -4009,7 +4049,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>278/0/0/0/0</t>
+          <t>278/0</t>
         </is>
       </c>
     </row>
@@ -4039,7 +4079,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>274/21/0/0/0</t>
+          <t>274/21</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4131,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>281/35/0/0/0</t>
+          <t>281/35</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4161,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>274/193/0/0/0</t>
+          <t>274/193</t>
         </is>
       </c>
     </row>
@@ -4217,7 +4257,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>283/5/0/0/0</t>
+          <t>283/5</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4309,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>274/224/0/0/0</t>
+          <t>274/224</t>
         </is>
       </c>
     </row>
@@ -4299,7 +4339,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>283/52/0/0/0</t>
+          <t>283/52</t>
         </is>
       </c>
     </row>
@@ -4329,7 +4369,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>281/38/0/0/0</t>
+          <t>281/38</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4399,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>281/38/0/0/0</t>
+          <t>281/38</t>
         </is>
       </c>
     </row>
@@ -4389,7 +4429,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>274/33/0/0/0</t>
+          <t>274/33</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4503,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>277/13/0/0/0</t>
+          <t>277/13</t>
         </is>
       </c>
     </row>
@@ -4493,7 +4533,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>274/8/0/0/0</t>
+          <t>274/8</t>
         </is>
       </c>
     </row>
@@ -4633,7 +4673,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>283/75/0/0/0</t>
+          <t>283/75</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4703,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>283/24/0/0/0</t>
+          <t>283/24</t>
         </is>
       </c>
     </row>
@@ -4693,7 +4733,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>283/24/0/0/0</t>
+          <t>283/24</t>
         </is>
       </c>
     </row>
@@ -4767,7 +4807,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>274/92/0/0/0</t>
+          <t>274/92</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4837,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>276/56/0/0/0</t>
+          <t>276/56</t>
         </is>
       </c>
     </row>
@@ -4827,7 +4867,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>274/6/0/0/0</t>
+          <t>274/6</t>
         </is>
       </c>
     </row>
@@ -4857,7 +4897,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>281/35/0/0/0</t>
+          <t>281/35</t>
         </is>
       </c>
     </row>
@@ -4887,7 +4927,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>281/35/0/0/0</t>
+          <t>281/35</t>
         </is>
       </c>
     </row>
@@ -4917,7 +4957,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>281/35/0/0/0</t>
+          <t>281/35</t>
         </is>
       </c>
     </row>
@@ -4947,7 +4987,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>281/35/0/0/0</t>
+          <t>281/35</t>
         </is>
       </c>
     </row>
@@ -4977,7 +5017,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>281/35/0/0/0</t>
+          <t>281/35</t>
         </is>
       </c>
     </row>
@@ -5051,7 +5091,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>274/33/0/0/0</t>
+          <t>274/33</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5121,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>283/21/0/0/0</t>
+          <t>283/21</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5151,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>283/21/0/0/0</t>
+          <t>283/21</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5181,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>283/22/0/0/0</t>
+          <t>283/22</t>
         </is>
       </c>
     </row>
@@ -5171,7 +5211,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>283/22/0/0/0</t>
+          <t>283/22</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5241,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>283/22/0/0/0</t>
+          <t>283/22</t>
         </is>
       </c>
     </row>
@@ -5231,7 +5271,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>283/22/0/0/0</t>
+          <t>283/22</t>
         </is>
       </c>
     </row>
@@ -5261,7 +5301,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>283/22/0/0/0</t>
+          <t>283/22</t>
         </is>
       </c>
     </row>
@@ -5288,56 +5328,64 @@
       <c r="F156" s="3" t="inlineStr"/>
     </row>
     <row r="157">
-      <c r="A157" t="n">
+      <c r="A157" s="4" t="n">
         <v>540887</v>
       </c>
-      <c r="B157" t="inlineStr">
+      <c r="B157" s="4" t="inlineStr">
         <is>
           <t>Servicii de setare si conectare a BD la UNA.md/Contabilitate</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr">
+      <c r="C157" s="4" t="inlineStr">
         <is>
           <t>serv.</t>
         </is>
       </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>activ</t>
-        </is>
-      </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>— serviciu, fara grupa</t>
-        </is>
-      </c>
-      <c r="F157" t="inlineStr"/>
+      <c r="D157" s="4" t="inlineStr">
+        <is>
+          <t>activ</t>
+        </is>
+      </c>
+      <c r="E157" s="4" t="inlineStr">
+        <is>
+          <t>Diverse (import e-Factura)</t>
+        </is>
+      </c>
+      <c r="F157" s="4" t="inlineStr">
+        <is>
+          <t>274/257</t>
+        </is>
+      </c>
     </row>
     <row r="158">
-      <c r="A158" t="n">
+      <c r="A158" s="4" t="n">
         <v>540888</v>
       </c>
-      <c r="B158" t="inlineStr">
+      <c r="B158" s="4" t="inlineStr">
         <is>
           <t>Servicii de mentenanta UNA.md de tip A la UNA.md/Contabilitate</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr">
+      <c r="C158" s="4" t="inlineStr">
         <is>
           <t>serv.</t>
         </is>
       </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>activ</t>
-        </is>
-      </c>
-      <c r="E158" t="inlineStr">
-        <is>
-          <t>— serviciu, fara grupa</t>
-        </is>
-      </c>
-      <c r="F158" t="inlineStr"/>
+      <c r="D158" s="4" t="inlineStr">
+        <is>
+          <t>activ</t>
+        </is>
+      </c>
+      <c r="E158" s="4" t="inlineStr">
+        <is>
+          <t>Diverse (import e-Factura)</t>
+        </is>
+      </c>
+      <c r="F158" s="4" t="inlineStr">
+        <is>
+          <t>274/257</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -5365,7 +5413,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>281/7/0/0/0</t>
+          <t>281/7</t>
         </is>
       </c>
     </row>
@@ -5395,7 +5443,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>281/7/0/0/0</t>
+          <t>281/7</t>
         </is>
       </c>
     </row>
@@ -5425,7 +5473,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>281/7/0/0/0</t>
+          <t>281/7</t>
         </is>
       </c>
     </row>
@@ -5455,7 +5503,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>281/7/0/0/0</t>
+          <t>281/7</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5533,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>281/7/0/0/0</t>
+          <t>281/7</t>
         </is>
       </c>
     </row>
@@ -5515,7 +5563,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>281/7/0/0/0</t>
+          <t>281/7</t>
         </is>
       </c>
     </row>
@@ -5545,35 +5593,39 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>286/25/0/0/0</t>
+          <t>286/25</t>
         </is>
       </c>
     </row>
     <row r="166">
-      <c r="A166" t="n">
+      <c r="A166" s="4" t="n">
         <v>540896</v>
       </c>
-      <c r="B166" t="inlineStr">
+      <c r="B166" s="4" t="inlineStr">
         <is>
           <t>Inregistrarea (fiscalizarea) sistemelor informatice cu sau fara dispozitive electronice fara imprimanta fiscala in REECC</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr">
+      <c r="C166" s="4" t="inlineStr">
         <is>
           <t>serv.</t>
         </is>
       </c>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>activ</t>
-        </is>
-      </c>
-      <c r="E166" t="inlineStr">
-        <is>
-          <t>— serviciu, fara grupa</t>
-        </is>
-      </c>
-      <c r="F166" t="inlineStr"/>
+      <c r="D166" s="4" t="inlineStr">
+        <is>
+          <t>activ</t>
+        </is>
+      </c>
+      <c r="E166" s="4" t="inlineStr">
+        <is>
+          <t>Diverse (import e-Factura)</t>
+        </is>
+      </c>
+      <c r="F166" s="4" t="inlineStr">
+        <is>
+          <t>274/257</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -5601,7 +5653,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>278/0/0/0/0</t>
+          <t>278/0</t>
         </is>
       </c>
     </row>
@@ -5631,7 +5683,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>274/100/0/0/0</t>
+          <t>274/100</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5735,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>274/0/0/0/0</t>
+          <t>274/0</t>
         </is>
       </c>
     </row>
@@ -5757,7 +5809,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>283/3/0/0/0</t>
+          <t>283/3</t>
         </is>
       </c>
     </row>
@@ -5787,7 +5839,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>274/122/0/0/0</t>
+          <t>274/122</t>
         </is>
       </c>
     </row>
@@ -5839,7 +5891,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>283/73/0/0/0</t>
+          <t>283/73</t>
         </is>
       </c>
     </row>
@@ -5891,7 +5943,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>274/92/0/0/0</t>
+          <t>274/92</t>
         </is>
       </c>
     </row>
@@ -5921,7 +5973,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>274/6/0/0/0</t>
+          <t>274/6</t>
         </is>
       </c>
     </row>
@@ -5951,7 +6003,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>286/15/0/0/0</t>
+          <t>286/15</t>
         </is>
       </c>
     </row>
@@ -6003,7 +6055,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>286/22/0/0/0</t>
+          <t>286/22</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6085,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>286/22/0/0/0</t>
+          <t>286/22</t>
         </is>
       </c>
     </row>
@@ -6063,7 +6115,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>274/133/0/0/0</t>
+          <t>274/133</t>
         </is>
       </c>
     </row>
@@ -6137,35 +6189,39 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>274/126/0/0/0</t>
+          <t>274/126</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="A188" t="n">
+      <c r="A188" s="4" t="n">
         <v>540918</v>
       </c>
-      <c r="B188" t="inlineStr">
+      <c r="B188" s="4" t="inlineStr">
         <is>
           <t>Factura ser. AAY nr. 7307328-7307527</t>
         </is>
       </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>buc.</t>
-        </is>
-      </c>
-      <c r="D188" t="inlineStr">
-        <is>
-          <t>activ</t>
-        </is>
-      </c>
-      <c r="E188" t="inlineStr">
-        <is>
-          <t>— serviciu, fara grupa</t>
-        </is>
-      </c>
-      <c r="F188" t="inlineStr"/>
+      <c r="C188" s="4" t="inlineStr">
+        <is>
+          <t>buc.</t>
+        </is>
+      </c>
+      <c r="D188" s="4" t="inlineStr">
+        <is>
+          <t>activ</t>
+        </is>
+      </c>
+      <c r="E188" s="4" t="inlineStr">
+        <is>
+          <t>Diverse (import e-Factura)</t>
+        </is>
+      </c>
+      <c r="F188" s="4" t="inlineStr">
+        <is>
+          <t>274/257</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="3" t="n">
@@ -6212,30 +6268,34 @@
       <c r="F190" s="3" t="inlineStr"/>
     </row>
     <row r="191">
-      <c r="A191" t="n">
+      <c r="A191" s="4" t="n">
         <v>540921</v>
       </c>
-      <c r="B191" t="inlineStr">
+      <c r="B191" s="4" t="inlineStr">
         <is>
           <t>Fiscal Cloud Mobile</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>buc.</t>
-        </is>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>activ</t>
-        </is>
-      </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>— serviciu, fara grupa</t>
-        </is>
-      </c>
-      <c r="F191" t="inlineStr"/>
+      <c r="C191" s="4" t="inlineStr">
+        <is>
+          <t>buc.</t>
+        </is>
+      </c>
+      <c r="D191" s="4" t="inlineStr">
+        <is>
+          <t>activ</t>
+        </is>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>Diverse (import e-Factura)</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="inlineStr">
+        <is>
+          <t>274/257</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="3" t="n">
@@ -6285,7 +6345,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>286/8/0/0/0</t>
+          <t>286/8</t>
         </is>
       </c>
     </row>
@@ -6337,7 +6397,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>274/244/0/0/0</t>
+          <t>274/244</t>
         </is>
       </c>
     </row>
@@ -6389,7 +6449,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>274/8/0/0/0</t>
+          <t>274/8</t>
         </is>
       </c>
     </row>
@@ -6419,7 +6479,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>274/207/0/0/0</t>
+          <t>274/207</t>
         </is>
       </c>
     </row>
@@ -6625,7 +6685,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>274/29/0/0/0</t>
+          <t>274/29</t>
         </is>
       </c>
     </row>
@@ -6721,7 +6781,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>274/63/0/0/0</t>
+          <t>274/63</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6833,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>274/21/0/0/0</t>
+          <t>274/21</t>
         </is>
       </c>
     </row>
@@ -6825,7 +6885,7 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>274/136/0/0/0</t>
+          <t>274/136</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6915,7 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>274/29/0/0/0</t>
+          <t>274/29</t>
         </is>
       </c>
     </row>
@@ -6951,7 +7011,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>281/35/0/0/0</t>
+          <t>281/35</t>
         </is>
       </c>
     </row>
@@ -6981,7 +7041,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>274/164/0/0/0</t>
+          <t>274/164</t>
         </is>
       </c>
     </row>
@@ -7011,7 +7071,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>274/164/0/0/0</t>
+          <t>274/164</t>
         </is>
       </c>
     </row>
@@ -7063,7 +7123,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>274/62/0/0/0</t>
+          <t>274/62</t>
         </is>
       </c>
     </row>
@@ -7137,7 +7197,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>274/111/0/0/0</t>
+          <t>274/111</t>
         </is>
       </c>
     </row>
@@ -7211,7 +7271,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>283/48/0/0/0</t>
+          <t>283/48</t>
         </is>
       </c>
     </row>
@@ -7241,7 +7301,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>274/21/0/0/0</t>
+          <t>274/21</t>
         </is>
       </c>
     </row>
@@ -7293,7 +7353,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>281/35/0/0/0</t>
+          <t>281/35</t>
         </is>
       </c>
     </row>
@@ -7320,108 +7380,124 @@
       <c r="F234" s="3" t="inlineStr"/>
     </row>
     <row r="235">
-      <c r="A235" t="n">
+      <c r="A235" s="4" t="n">
         <v>540965</v>
       </c>
-      <c r="B235" t="inlineStr">
+      <c r="B235" s="4" t="inlineStr">
         <is>
           <t>Procesearea Schimb de date 1C:Сomert cu Amanunt - 1C:Contabilitate 3.0</t>
         </is>
       </c>
-      <c r="C235" t="inlineStr">
-        <is>
-          <t>buc.</t>
-        </is>
-      </c>
-      <c r="D235" t="inlineStr">
-        <is>
-          <t>activ</t>
-        </is>
-      </c>
-      <c r="E235" t="inlineStr">
-        <is>
-          <t>— serviciu, fara grupa</t>
-        </is>
-      </c>
-      <c r="F235" t="inlineStr"/>
+      <c r="C235" s="4" t="inlineStr">
+        <is>
+          <t>buc.</t>
+        </is>
+      </c>
+      <c r="D235" s="4" t="inlineStr">
+        <is>
+          <t>activ</t>
+        </is>
+      </c>
+      <c r="E235" s="4" t="inlineStr">
+        <is>
+          <t>Diverse (import e-Factura)</t>
+        </is>
+      </c>
+      <c r="F235" s="4" t="inlineStr">
+        <is>
+          <t>274/257</t>
+        </is>
+      </c>
     </row>
     <row r="236">
-      <c r="A236" t="n">
+      <c r="A236" s="4" t="n">
         <v>540966</v>
       </c>
-      <c r="B236" t="inlineStr">
+      <c r="B236" s="4" t="inlineStr">
         <is>
           <t>Cloud Gestionare 2 utilizatori / 12 luni</t>
         </is>
       </c>
-      <c r="C236" t="inlineStr">
-        <is>
-          <t>buc.</t>
-        </is>
-      </c>
-      <c r="D236" t="inlineStr">
-        <is>
-          <t>activ</t>
-        </is>
-      </c>
-      <c r="E236" t="inlineStr">
-        <is>
-          <t>— serviciu, fara grupa</t>
-        </is>
-      </c>
-      <c r="F236" t="inlineStr"/>
+      <c r="C236" s="4" t="inlineStr">
+        <is>
+          <t>buc.</t>
+        </is>
+      </c>
+      <c r="D236" s="4" t="inlineStr">
+        <is>
+          <t>activ</t>
+        </is>
+      </c>
+      <c r="E236" s="4" t="inlineStr">
+        <is>
+          <t>Diverse (import e-Factura)</t>
+        </is>
+      </c>
+      <c r="F236" s="4" t="inlineStr">
+        <is>
+          <t>274/257</t>
+        </is>
+      </c>
     </row>
     <row r="237">
-      <c r="A237" t="n">
+      <c r="A237" s="4" t="n">
         <v>540967</v>
       </c>
-      <c r="B237" t="inlineStr">
+      <c r="B237" s="4" t="inlineStr">
         <is>
           <t>Cloud Contabilitate / 12 luni</t>
         </is>
       </c>
-      <c r="C237" t="inlineStr">
-        <is>
-          <t>buc.</t>
-        </is>
-      </c>
-      <c r="D237" t="inlineStr">
-        <is>
-          <t>activ</t>
-        </is>
-      </c>
-      <c r="E237" t="inlineStr">
-        <is>
-          <t>— serviciu, fara grupa</t>
-        </is>
-      </c>
-      <c r="F237" t="inlineStr"/>
+      <c r="C237" s="4" t="inlineStr">
+        <is>
+          <t>buc.</t>
+        </is>
+      </c>
+      <c r="D237" s="4" t="inlineStr">
+        <is>
+          <t>activ</t>
+        </is>
+      </c>
+      <c r="E237" s="4" t="inlineStr">
+        <is>
+          <t>Diverse (import e-Factura)</t>
+        </is>
+      </c>
+      <c r="F237" s="4" t="inlineStr">
+        <is>
+          <t>274/257</t>
+        </is>
+      </c>
     </row>
     <row r="238">
-      <c r="A238" t="n">
+      <c r="A238" s="4" t="n">
         <v>540968</v>
       </c>
-      <c r="B238" t="inlineStr">
+      <c r="B238" s="4" t="inlineStr">
         <is>
           <t>Sincronizarea FiscalCloudMobile cu Gestionare</t>
         </is>
       </c>
-      <c r="C238" t="inlineStr">
-        <is>
-          <t>buc.</t>
-        </is>
-      </c>
-      <c r="D238" t="inlineStr">
-        <is>
-          <t>activ</t>
-        </is>
-      </c>
-      <c r="E238" t="inlineStr">
-        <is>
-          <t>— serviciu, fara grupa</t>
-        </is>
-      </c>
-      <c r="F238" t="inlineStr"/>
+      <c r="C238" s="4" t="inlineStr">
+        <is>
+          <t>buc.</t>
+        </is>
+      </c>
+      <c r="D238" s="4" t="inlineStr">
+        <is>
+          <t>activ</t>
+        </is>
+      </c>
+      <c r="E238" s="4" t="inlineStr">
+        <is>
+          <t>Diverse (import e-Factura)</t>
+        </is>
+      </c>
+      <c r="F238" s="4" t="inlineStr">
+        <is>
+          <t>274/257</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F238"/>
@@ -7430,6 +7506,769 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="66" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Denumirea</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Tip card</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Provenienta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>288769</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Caiet 24 foi patratele asortate Yalong 7024-87K</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>288784</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Caiet 48 foi patratele Yalong 7048-593K</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>288787</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Caiet 48 foi patratele flowers asorti Yalong 7048-587K</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>288790</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Caiet 48 foi linie asortate Yalong 7048-576L</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>288794</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Caiet 96 foi linie BG "Forest Wonder"</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>289105</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Suport pentru carti  beige 1219s-1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>290956</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Set carioci 10 cul. MARCO Ultra Washable 1690-10</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>301409</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Caiet 96 foi patratele BG "Feeling"</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>301502</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Suport de masa cu compartiment p/u blocuri de hirtie, din metal, tip plasa, argintie</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>301651</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Set din 4 pensule Pony,Kite, rotunde 2, 3, 4, 5 in penar</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>301801</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Biblioraft A4/50 mm, HELLO!, VERDE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>301805</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Biblioraft A4/50 mm, HELLO!, ALBASTRU</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>301806</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Biblioraft A4/50 mm, HELLO!, NEGRU</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>301825</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Set de suport-uri pentru documente 3 sectii, din metal, argintie</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>302822</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Set de invelitori pentru manuale clasa 5, scoli romane, art. H.3666</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>302824</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Set de invelitori pentru manuale clasa 7, scoli romane, art. H.3668</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>302825</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Set de invelitori pentru manuale clasa 8, scoli romane, art. H.3669</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>302935</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Capse №26/8, LUX, 1000 buc.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>303070</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Capse №24/6 OfficeLine (1000 bucati)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>486534</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Power Cord PC-220V 1.8m Russian Plug, High quality, Cablexpert, PC-184-VDE</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>540711</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Jurnal Cartea mare, forma J-18 A4, 100 foi, ofset alb</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>540712</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Formular Foaie liniata, A3, ofset alb, 100 bucati</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>540713</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Formular Bon de primire hirtie ofset, 100 buc.</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>540714</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Jurnal Registru de casa, CO-04, A4, 50 foi, ofset alb</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>exista de mai demult</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>540810</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Cloud Baza Storno</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>nou</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>540823</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Servicii de certificare a cheilor publice pentru semnatura electronica calificata cu termen de valabilitate 2 an</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>nou</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>540824</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Dispozitiv criptografic-ePass 2003</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>nou</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>540887</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Servicii de setare si conectare a BD la UNA.md/Contabilitate</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>nou</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>540888</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Servicii de mentenanta UNA.md de tip A la UNA.md/Contabilitate</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>nou</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>540896</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Inregistrarea (fiscalizarea) sistemelor informatice cu sau fara dispozitive electronice fara imprimanta fiscala in REECC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>nou</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>540918</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Factura ser. AAY nr. 7307328-7307527</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>nou</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>540921</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Fiscal Cloud Mobile</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>nou</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>540965</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Procesearea Schimb de date 1C:Сomert cu Amanunt - 1C:Contabilitate 3.0</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>nou</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>540966</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Cloud Gestionare 2 utilizatori / 12 luni</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>nou</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>540967</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Cloud Contabilitate / 12 luni</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>nou</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>540968</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Sincronizarea FiscalCloudMobile cu Gestionare</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>nou</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D37"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7445,10 +8284,10 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -7505,7 +8344,7 @@
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>Din ele cu card</t>
+          <t>Cu card</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
@@ -7557,7 +8396,9 @@
       <c r="J2" t="n">
         <v>4</v>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="n">
+        <v>4</v>
+      </c>
       <c r="L2" t="n">
         <v>197.8</v>
       </c>
@@ -7606,7 +8447,7 @@
         <v>2</v>
       </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
         <v>349.45</v>
@@ -7806,7 +8647,7 @@
         <v>52</v>
       </c>
       <c r="K7" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="L7" t="n">
         <v>13346.16</v>
@@ -7856,7 +8697,7 @@
         <v>32</v>
       </c>
       <c r="K8" t="n">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="L8" t="n">
         <v>1267.55</v>
@@ -8056,7 +8897,7 @@
         <v>8</v>
       </c>
       <c r="K12" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L12" t="n">
         <v>1982.24</v>
@@ -8106,7 +8947,7 @@
         <v>4</v>
       </c>
       <c r="K13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L13" t="n">
         <v>2304.2</v>
@@ -8155,7 +8996,9 @@
       <c r="J14" t="n">
         <v>1</v>
       </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
       <c r="L14" t="n">
         <v>24</v>
       </c>
@@ -8204,7 +9047,7 @@
         <v>8</v>
       </c>
       <c r="K15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L15" t="n">
         <v>534.98</v>
@@ -8253,7 +9096,9 @@
       <c r="J16" t="n">
         <v>1</v>
       </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
       <c r="L16" t="n">
         <v>-6500</v>
       </c>
@@ -8402,7 +9247,7 @@
         <v>3</v>
       </c>
       <c r="K19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L19" t="n">
         <v>484</v>
@@ -8451,7 +9296,9 @@
       <c r="J20" t="n">
         <v>2</v>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="n">
+        <v>2</v>
+      </c>
       <c r="L20" t="n">
         <v>485</v>
       </c>
@@ -8550,7 +9397,7 @@
         <v>6</v>
       </c>
       <c r="K22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L22" t="n">
         <v>943.95</v>
@@ -8850,7 +9697,7 @@
         <v>61</v>
       </c>
       <c r="K28" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L28" t="n">
         <v>3201.07</v>
@@ -8899,7 +9746,9 @@
       <c r="J29" t="n">
         <v>2</v>
       </c>
-      <c r="K29" t="inlineStr"/>
+      <c r="K29" t="n">
+        <v>2</v>
+      </c>
       <c r="L29" t="n">
         <v>7249.9</v>
       </c>
@@ -8997,7 +9846,9 @@
       <c r="J31" t="n">
         <v>1</v>
       </c>
-      <c r="K31" t="inlineStr"/>
+      <c r="K31" t="n">
+        <v>1</v>
+      </c>
       <c r="L31" t="n">
         <v>528.5</v>
       </c>
@@ -9096,7 +9947,7 @@
         <v>25</v>
       </c>
       <c r="K33" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="L33" t="n">
         <v>1006.29</v>
@@ -9295,7 +10146,9 @@
       <c r="J37" t="n">
         <v>1</v>
       </c>
-      <c r="K37" t="inlineStr"/>
+      <c r="K37" t="n">
+        <v>1</v>
+      </c>
       <c r="L37" t="n">
         <v>320</v>
       </c>
@@ -9443,7 +10296,9 @@
       <c r="J40" t="n">
         <v>1</v>
       </c>
-      <c r="K40" t="inlineStr"/>
+      <c r="K40" t="n">
+        <v>1</v>
+      </c>
       <c r="L40" t="n">
         <v>840</v>
       </c>
@@ -9491,7 +10346,9 @@
       <c r="J41" t="n">
         <v>2</v>
       </c>
-      <c r="K41" t="inlineStr"/>
+      <c r="K41" t="n">
+        <v>2</v>
+      </c>
       <c r="L41" t="n">
         <v>156</v>
       </c>
@@ -9540,7 +10397,7 @@
         <v>2</v>
       </c>
       <c r="K42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L42" t="n">
         <v>655.55</v>
@@ -9690,7 +10547,7 @@
         <v>9</v>
       </c>
       <c r="K45" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L45" t="n">
         <v>2938.15</v>
@@ -9740,7 +10597,7 @@
         <v>42</v>
       </c>
       <c r="K46" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="L46" t="n">
         <v>4008.67</v>
@@ -9790,7 +10647,7 @@
         <v>10</v>
       </c>
       <c r="K47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L47" t="n">
         <v>1388.29</v>
@@ -9839,7 +10696,9 @@
       <c r="J48" t="n">
         <v>4</v>
       </c>
-      <c r="K48" t="inlineStr"/>
+      <c r="K48" t="n">
+        <v>4</v>
+      </c>
       <c r="L48" t="n">
         <v>11000</v>
       </c>
@@ -9878,7 +10737,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>NU (deja introdusa: doc 4)</t>
+          <t>NU — deja introdusa (doc 4)</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>

</xml_diff>